<commit_message>
Sync mobile grades artifacts and void validator for 2026-05-08 after grader run.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-08.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-08.xlsx
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>8</v>
       </c>
       <c r="G3" t="n">
-        <v>52.9</v>
+        <v>55.6</v>
       </c>
     </row>
     <row r="4">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="E8" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F8" t="n">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="G8" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>168</v>
+        <v>228</v>
       </c>
       <c r="E9" t="n">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="F9" t="n">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="G9" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>590</v>
+        <v>603</v>
       </c>
       <c r="E10" t="n">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="F10" t="n">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G10" t="n">
-        <v>61.9</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>343</v>
+        <v>366</v>
       </c>
       <c r="E11" t="n">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="F11" t="n">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="G11" t="n">
-        <v>63.6</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="E12" t="n">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F12" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G12" t="n">
-        <v>62</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E13" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F13" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="G13" t="n">
-        <v>66.7</v>
+        <v>65.90000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="E14" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="F14" t="n">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="G14" t="n">
-        <v>23.1</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>124</v>
+        <v>173</v>
       </c>
       <c r="E15" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="G15" t="n">
-        <v>12.9</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="E16" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F16" t="n">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="G16" t="n">
-        <v>30.6</v>
+        <v>26.5</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2357</v>
+        <v>2376</v>
       </c>
       <c r="E17" t="n">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="F17" t="n">
-        <v>1867</v>
+        <v>1884</v>
       </c>
       <c r="G17" t="n">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
     </row>
   </sheetData>
@@ -1442,29 +1442,53 @@
           <t>Weak</t>
         </is>
       </c>
+      <c r="B6" t="n">
+        <v>71.40000000000001</v>
+      </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="D6" t="n">
+        <v>53.8</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>13</v>
+      </c>
+      <c r="F6" t="n">
+        <v>66.7</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="H6" t="n">
+        <v>66.7</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="J6" t="n">
+        <v>75</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>8</v>
+      </c>
+      <c r="L6" t="n">
+        <v>11.1</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>27</v>
+      </c>
+      <c r="N6" t="n">
+        <v>8.300000000000001</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>12</v>
+      </c>
+      <c r="P6" t="n">
+        <v>10</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -1475,8 +1499,11 @@
       <c r="W6" t="n">
         <v>0</v>
       </c>
+      <c r="X6" t="n">
+        <v>100</v>
+      </c>
       <c r="Y6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA6" t="n">
         <v>0</v>
@@ -1487,8 +1514,11 @@
       <c r="AE6" t="n">
         <v>0</v>
       </c>
+      <c r="AF6" t="n">
+        <v>51.2</v>
+      </c>
       <c r="AG6" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -1498,52 +1528,52 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>61.9</v>
+        <v>62.2</v>
       </c>
       <c r="C7" t="n">
-        <v>590</v>
+        <v>603</v>
       </c>
       <c r="D7" t="n">
-        <v>63.6</v>
+        <v>63.1</v>
       </c>
       <c r="E7" t="n">
-        <v>343</v>
+        <v>366</v>
       </c>
       <c r="F7" t="n">
-        <v>62</v>
+        <v>62.3</v>
       </c>
       <c r="G7" t="n">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="H7" t="n">
-        <v>66.7</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="J7" t="n">
-        <v>23.1</v>
+        <v>25.7</v>
       </c>
       <c r="K7" t="n">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="L7" t="n">
-        <v>12.9</v>
+        <v>13.3</v>
       </c>
       <c r="M7" t="n">
-        <v>124</v>
+        <v>173</v>
       </c>
       <c r="N7" t="n">
-        <v>30.6</v>
+        <v>26.5</v>
       </c>
       <c r="O7" t="n">
-        <v>62</v>
+        <v>83</v>
       </c>
       <c r="P7" t="n">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>2357</v>
+        <v>2376</v>
       </c>
       <c r="R7" t="n">
         <v>54.7</v>
@@ -1564,16 +1594,16 @@
         <v>35</v>
       </c>
       <c r="X7" t="n">
-        <v>46.5</v>
+        <v>46.4</v>
       </c>
       <c r="Y7" t="n">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="Z7" t="n">
-        <v>52.9</v>
+        <v>55.6</v>
       </c>
       <c r="AA7" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AB7" t="n">
         <v>51.2</v>
@@ -1588,10 +1618,10 @@
         <v>24</v>
       </c>
       <c r="AF7" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="AG7" t="n">
-        <v>168</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync slate and graded data, mobile www artifacts, site nav CSS, and pipeline scripts.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-08.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-08.xlsx
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" t="n">
         <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>58.3</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E8" t="n">
         <v>103</v>
       </c>
       <c r="F8" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G8" t="n">
-        <v>46.4</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="E9" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="F9" t="n">
         <v>115</v>
       </c>
       <c r="G9" t="n">
-        <v>49.6</v>
+        <v>50.2</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="E10" t="n">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F10" t="n">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="G10" t="n">
-        <v>62.2</v>
+        <v>61.4</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="E11" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F11" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G11" t="n">
-        <v>63.1</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E14" t="n">
         <v>37</v>
       </c>
       <c r="F14" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="G14" t="n">
-        <v>25.7</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E15" t="n">
         <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G15" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E16" t="n">
         <v>22</v>
       </c>
       <c r="F16" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G16" t="n">
-        <v>26.5</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2376</v>
+        <v>2430</v>
       </c>
       <c r="E17" t="n">
-        <v>492</v>
+        <v>498</v>
       </c>
       <c r="F17" t="n">
-        <v>1884</v>
+        <v>1932</v>
       </c>
       <c r="G17" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
     </row>
   </sheetData>
@@ -1528,16 +1528,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62.2</v>
+        <v>61.4</v>
       </c>
       <c r="C7" t="n">
-        <v>603</v>
+        <v>614</v>
       </c>
       <c r="D7" t="n">
-        <v>63.1</v>
+        <v>63</v>
       </c>
       <c r="E7" t="n">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="F7" t="n">
         <v>62.3</v>
@@ -1552,28 +1552,28 @@
         <v>185</v>
       </c>
       <c r="J7" t="n">
-        <v>25.7</v>
+        <v>25.2</v>
       </c>
       <c r="K7" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L7" t="n">
-        <v>13.3</v>
+        <v>13.2</v>
       </c>
       <c r="M7" t="n">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="N7" t="n">
-        <v>26.5</v>
+        <v>25.9</v>
       </c>
       <c r="O7" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="P7" t="n">
-        <v>20.7</v>
+        <v>20.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>2376</v>
+        <v>2430</v>
       </c>
       <c r="R7" t="n">
         <v>54.7</v>
@@ -1594,10 +1594,10 @@
         <v>35</v>
       </c>
       <c r="X7" t="n">
-        <v>46.4</v>
+        <v>46.2</v>
       </c>
       <c r="Y7" t="n">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Z7" t="n">
         <v>55.6</v>
@@ -1612,16 +1612,16 @@
         <v>43</v>
       </c>
       <c r="AD7" t="n">
-        <v>58.3</v>
+        <v>60</v>
       </c>
       <c r="AE7" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AF7" t="n">
-        <v>49.6</v>
+        <v>50.2</v>
       </c>
       <c r="AG7" t="n">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>